<commit_message>
fix: preserve urgent priorities through import and planning
</commit_message>
<xml_diff>
--- a/site/public/beego-orders-template.xlsx
+++ b/site/public/beego-orders-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заявки" sheetId="1" r:id="R9fd932a1f95c4cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пояснения" sheetId="2" r:id="R126e6e05df634b2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заявки" sheetId="1" r:id="R319c136c0b2b48d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пояснения" sheetId="2" r:id="R046ad8bd1aab4f4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -634,7 +634,7 @@
         <x:v>Диагностика</x:v>
       </x:c>
       <x:c r="P3" s="17" t="str">
-        <x:v>HIGH</x:v>
+        <x:v>URGENT</x:v>
       </x:c>
       <x:c r="Q3" s="17" t="str">
         <x:v>ANY</x:v>
@@ -12090,7 +12090,7 @@
       <x:formula2>1440</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="P2:P5000">
-      <x:formula1>"NORMAL,HIGH,EMERGENCY"</x:formula1>
+      <x:formula1>"NORMAL,URGENT"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Q2:Q5000">
       <x:formula1>"ANY,CAR,PUBLIC_TRANSIT,WALKING,BICYCLE"</x:formula1>
@@ -12287,7 +12287,7 @@
         <x:v>Приоритет</x:v>
       </x:c>
       <x:c r="D12" s="27" t="str">
-        <x:v>NORMAL / HIGH / EMERGENCY</x:v>
+        <x:v>NORMAL / URGENT</x:v>
       </x:c>
       <x:c r="E12" s="27" t="str">
         <x:v>NORMAL</x:v>

</xml_diff>

<commit_message>
feat: add scoped object complexity and authoritative visit durations
</commit_message>
<xml_diff>
--- a/site/public/beego-orders-template.xlsx
+++ b/site/public/beego-orders-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заявки" sheetId="1" r:id="Rb9e4de5820864d9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пояснения" sheetId="2" r:id="R5609c5158d984886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Заявки" sheetId="1" r:id="Ra799613624c644a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пояснения" sheetId="2" r:id="Rcd015622aaa54cab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -138,7 +138,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -228,6 +228,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -455,6 +458,10 @@
     <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="32" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="52" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="52" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="52" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -521,8 +528,20 @@
       <x:c r="U1" s="6" t="str">
         <x:v>notes</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2">
+      <x:c r="V1" s="6" t="str">
+        <x:v>duration_factors</x:v>
+      </x:c>
+      <x:c r="W1" s="6" t="str">
+        <x:v>duration_override</x:v>
+      </x:c>
+      <x:c r="X1" s="6" t="str">
+        <x:v>service_entities</x:v>
+      </x:c>
+      <x:c r="Y1" s="6" t="str">
+        <x:v>object_id</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="16" t="str">
         <x:v>JOB-0001</x:v>
       </x:c>
@@ -586,8 +605,14 @@
       <x:c r="U2" s="16" t="str">
         <x:v>Связаться за 30 минут</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3">
+      <x:c r="V2" s="16" t="str">
+        <x:v>{"line":"existing","devices":1}</x:v>
+      </x:c>
+      <x:c r="W2" s="16" t="str"/>
+      <x:c r="X2" s="16" t="str"/>
+      <x:c r="Y2" s="16" t="str"/>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="17" t="str">
         <x:v>JOB-0002</x:v>
       </x:c>
@@ -651,6 +676,12 @@
       <x:c r="U3" s="17" t="str">
         <x:v>Проверить линию и оборудование</x:v>
       </x:c>
+      <x:c r="V3" s="17" t="str">
+        <x:v>{"diagnosis":"intermittent","segments":2}</x:v>
+      </x:c>
+      <x:c r="W3" s="17" t="str"/>
+      <x:c r="X3" s="17" t="str"/>
+      <x:c r="Y3" s="17" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="12"/>
@@ -12370,6 +12401,96 @@
       <x:c r="D19" s="38"/>
       <x:c r="E19" s="39"/>
     </x:row>
+    <x:row r="20" ht="46" customHeight="1">
+      <x:c r="A20" s="27" t="str">
+        <x:v>duration_factors</x:v>
+      </x:c>
+      <x:c r="B20" s="27" t="str">
+        <x:v>Нет</x:v>
+      </x:c>
+      <x:c r="C20" s="27" t="str">
+        <x:v>Состав работ для автоматического расчёта</x:v>
+      </x:c>
+      <x:c r="D20" s="27" t="str">
+        <x:v>Объект JSON</x:v>
+      </x:c>
+      <x:c r="E20" s="27" t="str">
+        <x:v>{"line":"existing","devices":1}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="46" customHeight="1">
+      <x:c r="A21" s="28" t="str">
+        <x:v>duration_override</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="str">
+        <x:v>Нет</x:v>
+      </x:c>
+      <x:c r="C21" s="28" t="str">
+        <x:v>Явная ручная длительность с основанием</x:v>
+      </x:c>
+      <x:c r="D21" s="28" t="str">
+        <x:v>Объект JSON</x:v>
+      </x:c>
+      <x:c r="E21" s="28" t="str">
+        <x:v>{"minutes":85,"reason":"Дополнительная точка"}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="46" customHeight="1">
+      <x:c r="A22" t="str">
+        <x:v>service_entities</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Нет</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>Существующие ID из паспорта объекта</x:v>
+      </x:c>
+      <x:c r="D22" s="40" t="str">
+        <x:v>Объект JSON</x:v>
+      </x:c>
+      <x:c r="E22" s="40" t="str">
+        <x:v>{"object":"ID","node":"ID"}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="46" customHeight="1">
+      <x:c r="A23" t="str">
+        <x:v>object_id</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Нет</x:v>
+      </x:c>
+      <x:c r="C23" s="40" t="str">
+        <x:v>ID объекта из реестра BeeGo!</x:v>
+      </x:c>
+      <x:c r="D23" s="40" t="str">
+        <x:v>Текст</x:v>
+      </x:c>
+      <x:c r="E23" s="40" t="str">
+        <x:v>Если неизвестен, оставьте пустым</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="46" customHeight="1">
+      <x:c r="A24" t="str">
+        <x:v>Старые файлы</x:v>
+      </x:c>
+      <x:c r="B24" t="str"/>
+      <x:c r="C24" s="40" t="str">
+        <x:v>service_duration_min сохраняется как источник. Новый план рассчитывается сервером по виду работ; произвольное число из файла не становится нормативом.</x:v>
+      </x:c>
+      <x:c r="D24" s="40" t="str"/>
+      <x:c r="E24" s="40" t="str"/>
+    </x:row>
+    <x:row r="25" ht="46" customHeight="1">
+      <x:c r="A25" t="str">
+        <x:v>Единицы</x:v>
+      </x:c>
+      <x:c r="B25" t="str"/>
+      <x:c r="C25" s="40" t="str">
+        <x:v>Визит = техническая работа + оформление + подтверждённый дополнительный доступ. Дорога отдельно.</x:v>
+      </x:c>
+      <x:c r="D25" s="40" t="str"/>
+      <x:c r="E25" s="40" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>

</xml_diff>